<commit_message>
base en de excel de graficas
</commit_message>
<xml_diff>
--- a/Proyecto/Archivos de apoyo/indicadores_acceso_tecnologico cambios.xlsx
+++ b/Proyecto/Archivos de apoyo/indicadores_acceso_tecnologico cambios.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stefanivilleda/Desktop/Programación II/Proyecto/programa-II/Proyecto/output/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paulogarridogrijalva/Documents/GitHub/programa-II/Proyecto/Archivos de apoyo/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393F3E39-1B82-994F-8746-726C0554FEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65549B06-BDDB-E144-B3E4-B503069F48BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="indicadores_basicos" sheetId="1" r:id="rId1"/>
@@ -21,9 +21,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -268,7 +271,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0.0_-;\-* #,##0.0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -451,12 +454,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -469,13 +472,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -484,11 +487,11 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -497,12 +500,15 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -523,9 +529,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office 2013 - 2022">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -563,9 +569,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -598,26 +604,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -650,26 +639,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -980,8 +952,9 @@
       <c r="G4" s="20">
         <v>42.91</v>
       </c>
-      <c r="H4" s="20">
-        <v>79.430000000000007</v>
+      <c r="H4" s="24">
+        <f>+MAX(H5:H26)+_xlfn.STDEV.S(H5:H26)</f>
+        <v>200.00643246522139</v>
       </c>
       <c r="I4" s="21">
         <v>404.86327950600662</v>
@@ -1704,7 +1677,7 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B29" s="6">
-        <f t="shared" ref="B29:I29" si="0">MIN(B5:B26)</f>
+        <f t="shared" ref="B29:E29" si="0">MIN(B5:B26)</f>
         <v>21.62</v>
       </c>
       <c r="C29" s="6">
@@ -1739,7 +1712,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B30" s="6">
-        <f t="shared" ref="B30:I30" si="3">STDEV(B5:B26)</f>
+        <f t="shared" ref="B30:D30" si="3">STDEV(B5:B26)</f>
         <v>7.8238260809820712</v>
       </c>
       <c r="C30" s="6">

</xml_diff>